<commit_message>
Enhance deployment migration tool with status tracking and execution history
- Updated functions/scripts/deploy_migration.js and Python tool to record STATUS ('MIGRADO'/'ERROR') and LAST_DEPLOYED_AT timestamps in Excel
- Added history logging to functions/migration_history.log and functions/migration_history.json
- Enabled error resilience so script continues through the list if a deployment fails

Co-authored-by: EMTrvillatoro <99835179+EMTrvillatoro@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/functions/functions.xlsx
+++ b/functions/functions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:E93"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,6 +409,12 @@
       <c r="C1" t="str">
         <v>ENVIRONMENT</v>
       </c>
+      <c r="D1" t="str">
+        <v>STATUS</v>
+      </c>
+      <c r="E1" t="str">
+        <v>LAST_DEPLOYED_AT</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -420,6 +426,12 @@
       <c r="C2" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D2" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-10-15T00:13:44.766Z</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -431,6 +443,12 @@
       <c r="C3" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D3" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-10-15T00:13:44.793Z</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -442,6 +460,12 @@
       <c r="C4" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D4" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-10-15T00:13:44.808Z</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -453,6 +477,12 @@
       <c r="C5" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D5" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-10-15T00:13:44.824Z</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -464,6 +494,12 @@
       <c r="C6" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D6" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-10-15T00:13:44.839Z</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -475,6 +511,12 @@
       <c r="C7" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D7" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-10-15T00:13:44.853Z</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -486,6 +528,12 @@
       <c r="C8" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D8" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-10-15T00:13:44.865Z</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -497,6 +545,12 @@
       <c r="C9" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D9" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-10-15T00:13:44.870Z</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -508,6 +562,12 @@
       <c r="C10" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D10" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-10-15T00:13:44.877Z</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -519,6 +579,12 @@
       <c r="C11" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D11" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-10-15T00:13:44.884Z</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -530,6 +596,12 @@
       <c r="C12" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D12" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-10-15T00:13:44.890Z</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -541,6 +613,12 @@
       <c r="C13" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D13" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-10-15T00:13:44.896Z</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -552,6 +630,12 @@
       <c r="C14" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D14" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-10-15T00:13:44.904Z</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -563,6 +647,12 @@
       <c r="C15" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D15" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2026-10-15T00:13:44.916Z</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -574,6 +664,12 @@
       <c r="C16" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D16" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-10-15T00:13:44.926Z</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -585,6 +681,12 @@
       <c r="C17" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D17" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2026-10-15T00:13:44.932Z</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -596,6 +698,12 @@
       <c r="C18" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D18" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2026-10-15T00:13:44.935Z</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -607,6 +715,12 @@
       <c r="C19" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D19" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2026-10-15T00:13:44.939Z</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -618,6 +732,12 @@
       <c r="C20" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D20" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2026-10-15T00:13:44.942Z</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -629,6 +749,12 @@
       <c r="C21" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D21" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2026-10-15T00:13:44.945Z</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -640,6 +766,12 @@
       <c r="C22" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D22" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2026-10-15T00:13:44.949Z</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -651,6 +783,12 @@
       <c r="C23" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D23" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2026-10-15T00:13:44.952Z</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -662,6 +800,12 @@
       <c r="C24" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D24" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2026-10-15T00:13:44.957Z</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -673,6 +817,12 @@
       <c r="C25" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D25" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2026-10-15T00:13:44.960Z</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -684,6 +834,12 @@
       <c r="C26" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D26" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2026-10-15T00:13:44.963Z</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -695,6 +851,12 @@
       <c r="C27" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D27" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2026-10-15T00:13:44.967Z</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -706,6 +868,12 @@
       <c r="C28" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D28" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2026-10-15T00:13:44.970Z</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -717,6 +885,12 @@
       <c r="C29" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D29" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2026-10-15T00:13:44.974Z</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -728,6 +902,12 @@
       <c r="C30" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D30" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2026-10-15T00:13:44.978Z</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -739,6 +919,12 @@
       <c r="C31" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D31" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2026-10-15T00:13:44.982Z</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -750,6 +936,12 @@
       <c r="C32" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D32" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2026-10-15T00:13:44.987Z</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -761,6 +953,12 @@
       <c r="C33" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D33" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2026-10-15T00:13:44.992Z</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -772,6 +970,12 @@
       <c r="C34" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D34" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2026-10-15T00:13:44.997Z</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -783,6 +987,12 @@
       <c r="C35" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D35" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2026-10-15T00:13:45.002Z</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -794,6 +1004,12 @@
       <c r="C36" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D36" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2026-10-15T00:13:45.006Z</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -805,6 +1021,12 @@
       <c r="C37" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D37" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2026-10-15T00:13:45.010Z</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -816,6 +1038,12 @@
       <c r="C38" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D38" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2026-10-15T00:13:45.014Z</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -827,6 +1055,12 @@
       <c r="C39" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D39" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2026-10-15T00:13:45.021Z</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -838,6 +1072,12 @@
       <c r="C40" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D40" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E40" t="str">
+        <v>2026-10-15T00:13:45.025Z</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -849,6 +1089,12 @@
       <c r="C41" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D41" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E41" t="str">
+        <v>2026-10-15T00:13:45.029Z</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -860,6 +1106,12 @@
       <c r="C42" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D42" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E42" t="str">
+        <v>2026-10-15T00:13:45.033Z</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -871,6 +1123,12 @@
       <c r="C43" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D43" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E43" t="str">
+        <v>2026-10-15T00:13:45.036Z</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -882,6 +1140,12 @@
       <c r="C44" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D44" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E44" t="str">
+        <v>2026-10-15T00:13:45.040Z</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -893,6 +1157,12 @@
       <c r="C45" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D45" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E45" t="str">
+        <v>2026-10-15T00:13:45.044Z</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -904,6 +1174,12 @@
       <c r="C46" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D46" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E46" t="str">
+        <v>2026-10-15T00:13:45.048Z</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -915,6 +1191,12 @@
       <c r="C47" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D47" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E47" t="str">
+        <v>2026-10-15T00:13:45.052Z</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -926,6 +1208,12 @@
       <c r="C48" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D48" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E48" t="str">
+        <v>2026-10-15T00:13:45.055Z</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -937,6 +1225,12 @@
       <c r="C49" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D49" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E49" t="str">
+        <v>2026-10-15T00:13:45.059Z</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -948,6 +1242,12 @@
       <c r="C50" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D50" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2026-10-15T00:13:45.063Z</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -959,6 +1259,12 @@
       <c r="C51" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D51" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2026-10-15T00:13:45.066Z</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -970,6 +1276,12 @@
       <c r="C52" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D52" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E52" t="str">
+        <v>2026-10-15T00:13:45.070Z</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -981,6 +1293,12 @@
       <c r="C53" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D53" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E53" t="str">
+        <v>2026-10-15T00:13:45.073Z</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -992,6 +1310,12 @@
       <c r="C54" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D54" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E54" t="str">
+        <v>2026-10-15T00:13:45.077Z</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1003,6 +1327,12 @@
       <c r="C55" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D55" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E55" t="str">
+        <v>2026-10-15T00:13:45.081Z</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -1014,6 +1344,12 @@
       <c r="C56" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D56" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E56" t="str">
+        <v>2026-10-15T00:13:45.085Z</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -1025,6 +1361,12 @@
       <c r="C57" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D57" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E57" t="str">
+        <v>2026-10-15T00:13:45.088Z</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -1036,6 +1378,12 @@
       <c r="C58" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D58" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E58" t="str">
+        <v>2026-10-15T00:13:45.091Z</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -1047,6 +1395,12 @@
       <c r="C59" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D59" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E59" t="str">
+        <v>2026-10-15T00:13:45.096Z</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -1058,6 +1412,12 @@
       <c r="C60" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D60" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E60" t="str">
+        <v>2026-10-15T00:13:45.100Z</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -1069,6 +1429,12 @@
       <c r="C61" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D61" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E61" t="str">
+        <v>2026-10-15T00:13:45.105Z</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -1080,6 +1446,12 @@
       <c r="C62" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D62" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E62" t="str">
+        <v>2026-10-15T00:13:45.109Z</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -1091,6 +1463,12 @@
       <c r="C63" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D63" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E63" t="str">
+        <v>2026-10-15T00:13:45.112Z</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -1102,6 +1480,12 @@
       <c r="C64" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D64" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E64" t="str">
+        <v>2026-10-15T00:13:45.115Z</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -1113,6 +1497,12 @@
       <c r="C65" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D65" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E65" t="str">
+        <v>2026-10-15T00:13:45.118Z</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -1124,6 +1514,12 @@
       <c r="C66" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D66" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E66" t="str">
+        <v>2026-10-15T00:13:45.122Z</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -1135,6 +1531,12 @@
       <c r="C67" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D67" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E67" t="str">
+        <v>2026-10-15T00:13:45.125Z</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -1146,6 +1548,12 @@
       <c r="C68" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D68" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E68" t="str">
+        <v>2026-10-15T00:13:45.129Z</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -1157,6 +1565,12 @@
       <c r="C69" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D69" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E69" t="str">
+        <v>2026-10-15T00:13:45.132Z</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -1168,6 +1582,12 @@
       <c r="C70" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D70" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E70" t="str">
+        <v>2026-10-15T00:13:45.136Z</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -1179,6 +1599,12 @@
       <c r="C71" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D71" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E71" t="str">
+        <v>2026-10-15T00:13:45.139Z</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -1190,6 +1616,12 @@
       <c r="C72" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D72" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E72" t="str">
+        <v>2026-10-15T00:13:45.142Z</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -1201,6 +1633,12 @@
       <c r="C73" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D73" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E73" t="str">
+        <v>2026-10-15T00:13:45.146Z</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -1212,6 +1650,12 @@
       <c r="C74" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D74" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E74" t="str">
+        <v>2026-10-15T00:13:45.149Z</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -1223,6 +1667,12 @@
       <c r="C75" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D75" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E75" t="str">
+        <v>2026-10-15T00:13:45.154Z</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -1234,6 +1684,12 @@
       <c r="C76" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D76" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E76" t="str">
+        <v>2026-10-15T00:13:45.158Z</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -1245,6 +1701,12 @@
       <c r="C77" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D77" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E77" t="str">
+        <v>2026-10-15T00:13:45.161Z</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -1256,6 +1718,12 @@
       <c r="C78" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D78" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E78" t="str">
+        <v>2026-10-15T00:13:45.165Z</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -1267,6 +1735,12 @@
       <c r="C79" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D79" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E79" t="str">
+        <v>2026-10-15T00:13:45.168Z</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -1278,6 +1752,12 @@
       <c r="C80" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D80" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E80" t="str">
+        <v>2026-10-15T00:13:45.172Z</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -1289,6 +1769,12 @@
       <c r="C81" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D81" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E81" t="str">
+        <v>2026-10-15T00:13:45.175Z</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -1300,6 +1786,12 @@
       <c r="C82" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D82" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E82" t="str">
+        <v>2026-10-15T00:13:45.180Z</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -1311,6 +1803,12 @@
       <c r="C83" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D83" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E83" t="str">
+        <v>2026-10-15T00:13:45.183Z</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -1322,6 +1820,12 @@
       <c r="C84" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D84" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E84" t="str">
+        <v>2026-10-15T00:13:45.187Z</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -1333,6 +1837,12 @@
       <c r="C85" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D85" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E85" t="str">
+        <v>2026-10-15T00:13:45.190Z</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -1344,6 +1854,12 @@
       <c r="C86" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D86" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E86" t="str">
+        <v>2026-10-15T00:13:45.194Z</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -1355,6 +1871,12 @@
       <c r="C87" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D87" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E87" t="str">
+        <v>2026-10-15T00:13:45.197Z</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -1366,6 +1888,12 @@
       <c r="C88" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D88" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E88" t="str">
+        <v>2026-10-15T00:13:45.201Z</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -1377,6 +1905,12 @@
       <c r="C89" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D89" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E89" t="str">
+        <v>2026-10-15T00:13:45.205Z</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -1388,6 +1922,12 @@
       <c r="C90" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D90" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E90" t="str">
+        <v>2026-10-15T00:13:45.209Z</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -1399,6 +1939,12 @@
       <c r="C91" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D91" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E91" t="str">
+        <v>2026-10-15T00:13:45.213Z</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -1410,6 +1956,12 @@
       <c r="C92" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D92" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E92" t="str">
+        <v>2026-10-15T00:13:45.217Z</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -1421,10 +1973,16 @@
       <c r="C93" t="str">
         <v>2nd gen</v>
       </c>
+      <c r="D93" t="str">
+        <v>MIGRADO</v>
+      </c>
+      <c r="E93" t="str">
+        <v>2026-10-15T00:13:45.221Z</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E93"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>